<commit_message>
fix: gwp_total_total -> gwp_total
</commit_message>
<xml_diff>
--- a/translators/templates/translator_template_v2.0.0.xlsx
+++ b/translators/templates/translator_template_v2.0.0.xlsx
@@ -24166,12 +24166,12 @@
       <c r="A39" s="5" t="inlineStr"/>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>gwp_total_total</t>
+          <t>gwp_total</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Total Global Warming Potential - Total</t>
+          <t>Total Global Warming Potential</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: make project_country field required
</commit_message>
<xml_diff>
--- a/translators/templates/translator_template_v2.0.0.xlsx
+++ b/translators/templates/translator_template_v2.0.0.xlsx
@@ -127,7 +127,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="003592e3"/>
+        <fgColor rgb="0072b7ed"/>
       </patternFill>
     </fill>
     <fill>
@@ -137,12 +137,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0031658d"/>
+        <fgColor rgb="003592e3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="009dd2f3"/>
+        <fgColor rgb="00b8e0f7"/>
       </patternFill>
     </fill>
     <fill>
@@ -190,10 +190,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1"/>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1"/>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1"/>
@@ -219,10 +219,10 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="3"/>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="9"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="6"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="4"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="4"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="8"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="7"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="5"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="7"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="5"/>
   </cellXfs>
   <cellStyles count="14">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -10669,9 +10669,9 @@
           <t>Country</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>Strongly recommended</t>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: add some unknown enum variants
</commit_message>
<xml_diff>
--- a/translators/templates/translator_template_v2.0.0.xlsx
+++ b/translators/templates/translator_template_v2.0.0.xlsx
@@ -784,7 +784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -880,6 +880,21 @@
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5371,7 +5386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5468,6 +5483,21 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
     </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5479,7 +5509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5723,6 +5753,21 @@
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr"/>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15496,7 +15541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -15608,6 +15653,21 @@
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17318,7 +17378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -17449,6 +17509,21 @@
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr"/>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: add project phases and common phases
</commit_message>
<xml_diff>
--- a/translators/templates/translator_template_v2.0.0.xlsx
+++ b/translators/templates/translator_template_v2.0.0.xlsx
@@ -4690,7 +4690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5151,12 +5151,12 @@
       <c r="A30" s="5" t="inlineStr"/>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>GBDI_EndOfUse</t>
+          <t>LMVM_AT_LPH1_Grundlagenanalyse</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>GBDI_EndOfUse</t>
+          <t>LMVM_AT_LPH1_Grundlagenanalyse</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -5166,16 +5166,526 @@
       <c r="A31" s="5" t="inlineStr"/>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Other_National</t>
+          <t>LMVM_AT_LPH2_Vorentwurf</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Other_National</t>
+          <t>LMVM_AT_LPH2_Vorentwurf</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr"/>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>LMVM_AT_LPH3_Entwurfsplanung</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>LMVM_AT_LPH3_Entwurfsplanung</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr"/>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>LMVM_AT_LPH4_Einreichplanung</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>LMVM_AT_LPH4_Einreichplanung</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr"/>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>LMVM_AT_LPH5_Ausfuehrungsplanung</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>LMVM_AT_LPH5_Ausfuehrungsplanung</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr"/>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>LMVM_AT_LPH6_Ausschreibung</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>LMVM_AT_LPH6_Ausschreibung</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr"/>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>LMVM_AT_LPH7_BegleitungBauausfuehrung</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>LMVM_AT_LPH7_BegleitungBauausfuehrung</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr"/>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>LMVM_AT_LPH8_OertlicheBauaufsichtDokumentation</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>LMVM_AT_LPH8_OertlicheBauaufsichtDokumentation</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr"/>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>LMVM_AT_LPH9_Objektbetreuung</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>LMVM_AT_LPH9_Objektbetreuung</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr"/>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>MOP_FR_ESQ_Esquisse</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>MOP_FR_ESQ_Esquisse</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr"/>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>MOP_FR_DIAG_Diagnostic</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>MOP_FR_DIAG_Diagnostic</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr"/>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>MOP_FR_APS_AvantProjetSommaire</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>MOP_FR_APS_AvantProjetSommaire</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr"/>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>MOP_FR_APD_AvantProjetDefinitif</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>MOP_FR_APD_AvantProjetDefinitif</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr"/>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>MOP_FR_PRO_EtudesProjet</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>MOP_FR_PRO_EtudesProjet</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr"/>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>MOP_FR_ACT_AssistanceContratsTravaux</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>MOP_FR_ACT_AssistanceContratsTravaux</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr"/>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>MOP_FR_EXE_EtudesExecution</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>MOP_FR_EXE_EtudesExecution</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr"/>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>MOP_FR_VISA_VisaEtudesExecution</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>MOP_FR_VISA_VisaEtudesExecution</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr"/>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>MOP_FR_DET_DirectionExecutionTravaux</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>MOP_FR_DET_DirectionExecutionTravaux</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr"/>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>MOP_FR_AOR_AssistanceOperationsReception</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>MOP_FR_AOR_AssistanceOperationsReception</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr"/>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_1_InitiatiefHaalbaarheid</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_1_InitiatiefHaalbaarheid</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr"/>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_2_Projectdefinitie</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_2_Projectdefinitie</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr"/>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_3_Structuurontwerp</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_3_Structuurontwerp</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr"/>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_4_Voorontwerp</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_4_Voorontwerp</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr"/>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_5_DefinitiefOntwerp</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_5_DefinitiefOntwerp</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr"/>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_6_TechnischOntwerpBestek</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_6_TechnischOntwerpBestek</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr"/>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_7_PrijsEnContractvorming</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_7_PrijsEnContractvorming</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr"/>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_8_UitvoeringsgereedOntwerp</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_8_UitvoeringsgereedOntwerp</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr"/>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_9_Directievoering</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_9_Directievoering</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr"/>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_10_GebruikExploitatie</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>DNRSTB_NL_10_GebruikExploitatie</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr"/>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>LOE_ES_EP_EstudiosPrevios</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>LOE_ES_EP_EstudiosPrevios</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr"/>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>LOE_ES_AP_Anteproyecto</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>LOE_ES_AP_Anteproyecto</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr"/>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>LOE_ES_PB_ProyectoBasico</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>LOE_ES_PB_ProyectoBasico</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr"/>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>LOE_ES_PE_ProyectoEjecucion</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>LOE_ES_PE_ProyectoEjecucion</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr"/>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>LOE_ES_DO_DireccionObra</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>LOE_ES_DO_DireccionObra</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr"/>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>GBDI_EndOfUse</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>GBDI_EndOfUse</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr"/>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>Other_National</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>Other_National</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5349,12 +5859,12 @@
       <c r="A10" s="5" t="inlineStr"/>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>8 End of use, re-cycling</t>
+          <t>8 End of use, recycling</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>8 End of use, re-cycling</t>
+          <t>8 End of use, recycling</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>

</xml_diff>